<commit_message>
idek basically done with functionalities
</commit_message>
<xml_diff>
--- a/entity_plans/100 STATE DEPARTMENT FOR BASIC EDUCATION.xlsx
+++ b/entity_plans/100 STATE DEPARTMENT FOR BASIC EDUCATION.xlsx
@@ -97,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -105,11 +105,24 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,14 +491,14 @@
   <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="75" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="114" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -541,576 +554,1196 @@
       <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Paper Materials &amp; Products</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>4418366</v>
       </c>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr"/>
-      <c r="H3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Manufacturing Components &amp; Supplies</t>
         </is>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="5" t="n">
         <v>126920</v>
       </c>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr"/>
-      <c r="F4" s="3" t="inlineStr"/>
-      <c r="G4" s="3" t="inlineStr"/>
-      <c r="H4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Office Equipment &amp; Accessories &amp; Supplies</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>11614973.8</v>
       </c>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
-      <c r="H5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Musical Instruments &amp; Games &amp; Toys &amp; Arts &amp; Crafts &amp; Educational Equipment &amp; Materials &amp; Accessories &amp; Supplies</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <v>118176</v>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr"/>
-      <c r="F6" s="3" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr"/>
-      <c r="H6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Apparel &amp; Luggage &amp; Personal Care Products</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>857772</v>
       </c>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr"/>
-      <c r="H7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Published Products</t>
         </is>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="5" t="n">
         <v>263283.5</v>
       </c>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="3" t="inlineStr"/>
-      <c r="G8" s="3" t="inlineStr"/>
-      <c r="H8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Public Utilities &amp; Public Sector Related Services</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>15474172</v>
       </c>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="3" t="inlineStr"/>
-      <c r="G9" s="3" t="inlineStr"/>
-      <c r="H9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Engineering &amp; Research &amp; Technology Based Services</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
+      <c r="C10" s="5" t="n">
         <v>440493</v>
       </c>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="3" t="inlineStr"/>
-      <c r="G10" s="3" t="inlineStr"/>
-      <c r="H10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Transportation &amp; Storage &amp; Mail Services</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="5" t="n">
         <v>57837657</v>
       </c>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr"/>
-      <c r="H11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Editorial &amp; Design &amp; Graphic &amp; Fine Art Services</t>
         </is>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="C12" s="5" t="n">
         <v>539263</v>
       </c>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="inlineStr"/>
-      <c r="H12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Education &amp; Training Services</t>
         </is>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="C13" s="5" t="n">
         <v>1504221</v>
       </c>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr"/>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="inlineStr"/>
-      <c r="H13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Travel &amp; Food &amp; Lodging &amp; Entertainment Services</t>
         </is>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="C14" s="5" t="n">
         <v>39433061</v>
       </c>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr"/>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="inlineStr"/>
-      <c r="H14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Commercial &amp; Military &amp; Private Vehicles &amp; their Accessories &amp; Components</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="C15" s="5" t="n">
         <v>6501546</v>
       </c>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr"/>
-      <c r="F15" s="3" t="inlineStr"/>
-      <c r="G15" s="3" t="inlineStr"/>
-      <c r="H15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Power Generation &amp; Distribution Machinery &amp; Accessories</t>
         </is>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="5" t="n">
         <v>618324</v>
       </c>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr"/>
-      <c r="F16" s="3" t="inlineStr"/>
-      <c r="G16" s="3" t="inlineStr"/>
-      <c r="H16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Furniture &amp; Furnishings</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="C17" s="5" t="n">
         <v>467874</v>
       </c>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr"/>
-      <c r="F17" s="3" t="inlineStr"/>
-      <c r="G17" s="3" t="inlineStr"/>
-      <c r="H17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Building &amp; Construction &amp; Maintenance Services</t>
         </is>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="5" t="n">
         <v>1498374</v>
       </c>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr"/>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
-      <c r="H18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Electrical systems &amp; Lighting &amp; components &amp; accessories &amp; supplies</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="C19" s="5" t="n">
         <v>135190</v>
       </c>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr"/>
-      <c r="F19" s="3" t="inlineStr"/>
-      <c r="G19" s="3" t="inlineStr"/>
-      <c r="H19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>Information Technology Broadcasting &amp; Telecommunications</t>
         </is>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="5" t="n">
         <v>1209930</v>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr"/>
-      <c r="F20" s="3" t="inlineStr"/>
-      <c r="G20" s="3" t="inlineStr"/>
-      <c r="H20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ YOUTH/RFQ PWD</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>RFQ/RFQ WOMEN/RFQ PWD</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Fuels &amp; Fuel Additives &amp; Lubricants &amp; Anti corrosive Materials</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="5" t="n">
         <v>14702394</v>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr"/>
-      <c r="H21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>Industrial Production &amp; Manufacturing Services</t>
         </is>
       </c>
-      <c r="C22" s="4" t="n">
+      <c r="C22" s="5" t="n">
         <v>1806948</v>
       </c>
-      <c r="D22" s="3" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr"/>
-      <c r="F22" s="3" t="inlineStr"/>
-      <c r="G22" s="3" t="inlineStr"/>
-      <c r="H22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>RFQ</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Laboratory &amp; Measuring &amp; Observing &amp; Testing Equipment</t>
         </is>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="C23" s="5" t="n">
         <v>11801</v>
       </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
-      <c r="F23" s="3" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr"/>
-      <c r="H23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Tools &amp; General Machinery</t>
         </is>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="C24" s="5" t="n">
         <v>2400</v>
       </c>
-      <c r="D24" s="3" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr"/>
-      <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr"/>
-      <c r="H24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Service Industry Machinery &amp; Equipment &amp; Supplies</t>
         </is>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C25" s="5" t="n">
         <v>80700</v>
       </c>
-      <c r="D25" s="3" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr"/>
-      <c r="F25" s="3" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr"/>
-      <c r="H25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>Management &amp; Business Professionals &amp; Administrative Services</t>
         </is>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C26" s="5" t="n">
         <v>3281216</v>
       </c>
-      <c r="D26" s="3" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr"/>
-      <c r="F26" s="3" t="inlineStr"/>
-      <c r="G26" s="3" t="inlineStr"/>
-      <c r="H26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Defense &amp; Law Enforcement &amp; Security &amp; Safety Equipment &amp; Supplies</t>
         </is>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="C27" s="5" t="n">
         <v>544874</v>
       </c>
-      <c r="D27" s="3" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr"/>
-      <c r="F27" s="3" t="inlineStr"/>
-      <c r="G27" s="3" t="inlineStr"/>
-      <c r="H27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Material Handling &amp; Conditioning &amp; Storage Machinery &amp; their Accessories &amp; Supplies</t>
         </is>
       </c>
-      <c r="C28" s="4" t="n">
+      <c r="C28" s="5" t="n">
         <v>2500</v>
       </c>
-      <c r="D28" s="3" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr"/>
-      <c r="F28" s="3" t="inlineStr"/>
-      <c r="G28" s="3" t="inlineStr"/>
-      <c r="H28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Cleaning Equipment &amp; Supplies</t>
         </is>
       </c>
-      <c r="C29" s="4" t="n">
+      <c r="C29" s="5" t="n">
         <v>143050</v>
       </c>
-      <c r="D29" s="3" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="inlineStr"/>
-      <c r="H29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Industrial Manufacturing &amp; Processing Machinery &amp; Accessories</t>
         </is>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="C30" s="5" t="n">
         <v>10000</v>
       </c>
-      <c r="D30" s="3" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="3" t="inlineStr"/>
-      <c r="G30" s="3" t="inlineStr"/>
-      <c r="H30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Chemicals including Bio Chemicals &amp; Gas Materials</t>
         </is>
       </c>
-      <c r="C31" s="4" t="n">
+      <c r="C31" s="5" t="n">
         <v>82250</v>
       </c>
-      <c r="D31" s="3" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="3" t="inlineStr"/>
-      <c r="G31" s="3" t="inlineStr"/>
-      <c r="H31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN/RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Industrial Cleaning Services</t>
         </is>
       </c>
-      <c r="C32" s="4" t="n">
+      <c r="C32" s="5" t="n">
         <v>13260000</v>
       </c>
-      <c r="D32" s="3" t="inlineStr"/>
-      <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="3" t="inlineStr"/>
-      <c r="G32" s="3" t="inlineStr"/>
-      <c r="H32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>RFQ YOUTH</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
         <v>31</v>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Printing &amp; Photographic &amp; Audio &amp; Visual Equipment &amp; Supplies</t>
         </is>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C33" s="5" t="n">
         <v>200000</v>
       </c>
-      <c r="D33" s="3" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="3" t="inlineStr"/>
-      <c r="G33" s="3" t="inlineStr"/>
-      <c r="H33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>RFQ AGPO</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>RFQ WOMEN</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="7">
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="8">
         <f>SUM(C3:C33)</f>
         <v/>
       </c>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
+      <c r="D34" s="7" t="n"/>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="G34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>